<commit_message>
Update invoice data and regenerate source
Correct multiple TEXTBOOKS entries and corresponding grandTotal values in docs/data/invoice.json. Refresh docs/data/meta.json generatedAt timestamp and replace source/INVOICE.xlsx with the regenerated spreadsheet so the source and metadata reflect the corrected invoice data.
</commit_message>
<xml_diff>
--- a/source/INVOICE.xlsx
+++ b/source/INVOICE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\ADMISSION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CF95A7-79BB-4346-9015-0ECA4F51626E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBBB50F5-D031-4E6B-9A8F-F15437FABC71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="8">
-        <v>12360</v>
+        <v>12240</v>
       </c>
       <c r="I4" s="10">
         <v>7550</v>
@@ -742,7 +742,7 @@
       </c>
       <c r="Q4" s="17">
         <f t="shared" si="0"/>
-        <v>89910</v>
+        <v>89790</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="8">
-        <v>12840</v>
+        <v>13080</v>
       </c>
       <c r="I5" s="10">
         <v>7550</v>
@@ -796,7 +796,7 @@
       </c>
       <c r="Q5" s="17">
         <f t="shared" si="0"/>
-        <v>90390</v>
+        <v>90630</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -822,7 +822,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="8">
-        <v>28080</v>
+        <v>24870</v>
       </c>
       <c r="I6" s="10">
         <v>10730</v>
@@ -850,7 +850,7 @@
       </c>
       <c r="Q6" s="17">
         <f t="shared" si="0"/>
-        <v>108810</v>
+        <v>105600</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -876,7 +876,7 @@
         <v>5000</v>
       </c>
       <c r="H7" s="8">
-        <v>24900</v>
+        <v>25890</v>
       </c>
       <c r="I7" s="10">
         <v>11330</v>
@@ -904,7 +904,7 @@
       </c>
       <c r="Q7" s="17">
         <f t="shared" si="0"/>
-        <v>114730</v>
+        <v>115720</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -930,7 +930,7 @@
         <v>5000</v>
       </c>
       <c r="H8" s="8">
-        <v>24900</v>
+        <v>25890</v>
       </c>
       <c r="I8" s="10">
         <v>11330</v>
@@ -958,7 +958,7 @@
       </c>
       <c r="Q8" s="17">
         <f t="shared" si="0"/>
-        <v>114730</v>
+        <v>115720</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -984,7 +984,7 @@
         <v>5000</v>
       </c>
       <c r="H9" s="8">
-        <v>26040</v>
+        <v>27030</v>
       </c>
       <c r="I9" s="10">
         <v>13230</v>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="Q9" s="17">
         <f t="shared" si="0"/>
-        <v>117770</v>
+        <v>118760</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1038,7 +1038,7 @@
         <v>5000</v>
       </c>
       <c r="H10" s="8">
-        <v>26040</v>
+        <v>27030</v>
       </c>
       <c r="I10" s="10">
         <v>13230</v>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="Q10" s="17">
         <f t="shared" si="0"/>
-        <v>117770</v>
+        <v>118760</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
@@ -1092,7 +1092,7 @@
         <v>5000</v>
       </c>
       <c r="H11" s="8">
-        <v>27660</v>
+        <v>28890</v>
       </c>
       <c r="I11" s="10">
         <v>13230</v>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="Q11" s="17">
         <f t="shared" si="0"/>
-        <v>119390</v>
+        <v>120620</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1146,7 +1146,7 @@
         <v>6000</v>
       </c>
       <c r="H12" s="8">
-        <v>17940</v>
+        <v>19560</v>
       </c>
       <c r="I12" s="10">
         <v>16190</v>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="Q12" s="17">
         <f t="shared" si="0"/>
-        <v>119130</v>
+        <v>120750</v>
       </c>
     </row>
     <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1200,7 +1200,7 @@
         <v>6000</v>
       </c>
       <c r="H13" s="8">
-        <v>17940</v>
+        <v>19560</v>
       </c>
       <c r="I13" s="10">
         <v>14330</v>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="Q13" s="17">
         <f t="shared" si="0"/>
-        <v>117270</v>
+        <v>118890</v>
       </c>
     </row>
     <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1254,7 +1254,7 @@
         <v>6000</v>
       </c>
       <c r="H14" s="8">
-        <v>24180</v>
+        <v>22580</v>
       </c>
       <c r="I14" s="10">
         <v>14330</v>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="Q14" s="17">
         <f t="shared" si="0"/>
-        <v>123510</v>
+        <v>121910</v>
       </c>
     </row>
     <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1308,7 +1308,7 @@
         <v>8000</v>
       </c>
       <c r="H15" s="8">
-        <v>12480</v>
+        <v>14280</v>
       </c>
       <c r="I15" s="10">
         <v>14330</v>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="Q15" s="17">
         <f t="shared" si="0"/>
-        <v>128810</v>
+        <v>130610</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1362,7 +1362,7 @@
         <v>8000</v>
       </c>
       <c r="H16" s="8">
-        <v>12480</v>
+        <v>14280</v>
       </c>
       <c r="I16" s="10">
         <v>14330</v>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="Q16" s="17">
         <f t="shared" si="0"/>
-        <v>128810</v>
+        <v>130610</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1416,7 +1416,7 @@
         <v>8000</v>
       </c>
       <c r="H17" s="8">
-        <v>12480</v>
+        <v>14280</v>
       </c>
       <c r="I17" s="10">
         <v>14330</v>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="Q17" s="17">
         <f t="shared" si="0"/>
-        <v>128810</v>
+        <v>130610</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update fees, student balances and add .gitignore
Adjust fee data across docs/data (invoice.json, students.json, meta.json) to correct TEXTBOOKS values and recompute grand totals, student balances, and overall outstanding/summary counts. Replace multiple source Excel fee files (2022–2027) with updated versions. Add .gitignore to exclude __pycache__, .pyc, editor files and temporary Excel lock files (~$*.xlsx). Ensures JSON data stays consistent with updated spreadsheets and overall school fee/state totals.
</commit_message>
<xml_diff>
--- a/source/INVOICE.xlsx
+++ b/source/INVOICE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\ADMISSION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBBB50F5-D031-4E6B-9A8F-F15437FABC71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F1B7E6-8B59-418F-9DCC-CB423CA67BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,7 +660,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="8">
-        <v>8040</v>
+        <v>6840</v>
       </c>
       <c r="I3" s="10">
         <v>5300</v>
@@ -688,7 +688,7 @@
       </c>
       <c r="Q3" s="17">
         <f t="shared" si="0"/>
-        <v>83340</v>
+        <v>82140</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="8">
-        <v>12240</v>
+        <v>12480</v>
       </c>
       <c r="I4" s="10">
         <v>7550</v>
@@ -742,7 +742,7 @@
       </c>
       <c r="Q4" s="17">
         <f t="shared" si="0"/>
-        <v>89790</v>
+        <v>90030</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="8">
-        <v>13080</v>
+        <v>13380</v>
       </c>
       <c r="I5" s="10">
         <v>7550</v>
@@ -796,7 +796,7 @@
       </c>
       <c r="Q5" s="17">
         <f t="shared" si="0"/>
-        <v>90630</v>
+        <v>90930</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -822,7 +822,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="8">
-        <v>24870</v>
+        <v>24450</v>
       </c>
       <c r="I6" s="10">
         <v>10730</v>
@@ -850,7 +850,7 @@
       </c>
       <c r="Q6" s="17">
         <f t="shared" si="0"/>
-        <v>105600</v>
+        <v>105180</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -876,7 +876,7 @@
         <v>5000</v>
       </c>
       <c r="H7" s="8">
-        <v>25890</v>
+        <v>25550</v>
       </c>
       <c r="I7" s="10">
         <v>11330</v>
@@ -904,7 +904,7 @@
       </c>
       <c r="Q7" s="17">
         <f t="shared" si="0"/>
-        <v>115720</v>
+        <v>115380</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -930,7 +930,7 @@
         <v>5000</v>
       </c>
       <c r="H8" s="8">
-        <v>25890</v>
+        <v>25730</v>
       </c>
       <c r="I8" s="10">
         <v>11330</v>
@@ -958,7 +958,7 @@
       </c>
       <c r="Q8" s="17">
         <f t="shared" si="0"/>
-        <v>115720</v>
+        <v>115560</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -984,7 +984,7 @@
         <v>5000</v>
       </c>
       <c r="H9" s="8">
-        <v>27030</v>
+        <v>26890</v>
       </c>
       <c r="I9" s="10">
         <v>13230</v>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="Q9" s="17">
         <f t="shared" si="0"/>
-        <v>118760</v>
+        <v>118620</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1038,7 +1038,7 @@
         <v>5000</v>
       </c>
       <c r="H10" s="8">
-        <v>27030</v>
+        <v>26910</v>
       </c>
       <c r="I10" s="10">
         <v>13230</v>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="Q10" s="17">
         <f t="shared" si="0"/>
-        <v>118760</v>
+        <v>118640</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
@@ -1092,7 +1092,7 @@
         <v>5000</v>
       </c>
       <c r="H11" s="8">
-        <v>28890</v>
+        <v>28850</v>
       </c>
       <c r="I11" s="10">
         <v>13230</v>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="Q11" s="17">
         <f t="shared" si="0"/>
-        <v>120620</v>
+        <v>120580</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1308,7 +1308,7 @@
         <v>8000</v>
       </c>
       <c r="H15" s="8">
-        <v>14280</v>
+        <v>11880</v>
       </c>
       <c r="I15" s="10">
         <v>14330</v>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="Q15" s="17">
         <f t="shared" si="0"/>
-        <v>130610</v>
+        <v>128210</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1362,7 +1362,7 @@
         <v>8000</v>
       </c>
       <c r="H16" s="8">
-        <v>14280</v>
+        <v>11880</v>
       </c>
       <c r="I16" s="10">
         <v>14330</v>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="Q16" s="17">
         <f t="shared" si="0"/>
-        <v>130610</v>
+        <v>128210</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1416,7 +1416,7 @@
         <v>8000</v>
       </c>
       <c r="H17" s="8">
-        <v>14280</v>
+        <v>11880</v>
       </c>
       <c r="I17" s="10">
         <v>14330</v>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="Q17" s="17">
         <f t="shared" si="0"/>
-        <v>130610</v>
+        <v>128210</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>